<commit_message>
Actualitzar relació entre RA, CAs i Continguts
</commit_message>
<xml_diff>
--- a/_recursos_originals/2º DAW DWEC - RA i CA.xlsx
+++ b/_recursos_originals/2º DAW DWEC - RA i CA.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="28827"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29929"/>
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://upvedues.sharepoint.com/sites/TreballTecnologiaiDigitalitzaci/Documentos compartidos/General/_DIDÀCTICA 2/KARMA/"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Sofia\Git\_Karma\_recursos_originals\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="542" documentId="13_ncr:1_{EFE1F849-2408-4321-8631-716AF009FAB9}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{028066B3-99B5-43E4-A6FB-91FA4A6AE2CE}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{518AC857-55DC-45CF-937E-F66B3C443A9F}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{5DAFA8AD-9D14-4E79-BCEE-E5648B38B0AF}"/>
+    <workbookView xWindow="28680" yWindow="-3180" windowWidth="29040" windowHeight="15720" xr2:uid="{5DAFA8AD-9D14-4E79-BCEE-E5648B38B0AF}"/>
   </bookViews>
   <sheets>
     <sheet name="RA_CE" sheetId="1" r:id="rId1"/>
@@ -336,7 +336,7 @@
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="7" x14ac:knownFonts="1">
+  <fonts count="11" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -345,52 +345,70 @@
       <scheme val="minor"/>
     </font>
     <font>
+      <sz val="11"/>
+      <color theme="1"/>
+      <name val="Aptos"/>
+      <family val="2"/>
+    </font>
+    <font>
+      <sz val="12"/>
+      <color theme="0"/>
+      <name val="Aptos"/>
+      <family val="2"/>
+    </font>
+    <font>
       <b/>
       <sz val="11"/>
       <color theme="1"/>
-      <name val="Aptos Narrow"/>
+      <name val="Aptos"/>
       <family val="2"/>
-      <scheme val="minor"/>
+    </font>
+    <font>
+      <b/>
+      <sz val="12"/>
+      <color rgb="FF000000"/>
+      <name val="Aptos"/>
+      <family val="2"/>
+    </font>
+    <font>
+      <sz val="12"/>
+      <color rgb="FF000000"/>
+      <name val="Aptos"/>
+      <family val="2"/>
+    </font>
+    <font>
+      <sz val="12"/>
+      <color theme="1"/>
+      <name val="Aptos"/>
+      <family val="2"/>
     </font>
     <font>
       <b/>
       <sz val="11"/>
       <color rgb="FF000000"/>
-      <name val="Aptos Narrow"/>
+      <name val="Aptos"/>
       <family val="2"/>
-      <scheme val="minor"/>
     </font>
     <font>
       <sz val="11"/>
       <color rgb="FF000000"/>
-      <name val="Aptos Narrow"/>
+      <name val="Aptos"/>
       <family val="2"/>
-      <scheme val="minor"/>
     </font>
     <font>
-      <b/>
-      <sz val="12"/>
+      <sz val="16"/>
       <color theme="0"/>
-      <name val="Aptos Narrow"/>
+      <name val="Aptos"/>
       <family val="2"/>
-      <scheme val="minor"/>
     </font>
     <font>
-      <sz val="12"/>
-      <color theme="0"/>
-      <name val="Aptos Narrow"/>
+      <sz val="16"/>
+      <color theme="1"/>
+      <name val="Aptos"/>
       <family val="2"/>
-      <scheme val="minor"/>
-    </font>
-    <font>
-      <sz val="12"/>
-      <color theme="1"/>
-      <name val="Aptos Narrow"/>
-      <family val="2"/>
-      <scheme val="minor"/>
     </font>
   </fonts>
-  <fills count="5">
+  <fills count="4">
     <fill>
       <patternFill patternType="none"/>
     </fill>
@@ -409,14 +427,8 @@
         <bgColor indexed="64"/>
       </patternFill>
     </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor theme="0"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
   </fills>
-  <borders count="33">
+  <borders count="38">
     <border>
       <left/>
       <right/>
@@ -543,252 +555,90 @@
       <diagonal/>
     </border>
     <border>
+      <left style="medium">
+        <color indexed="64"/>
+      </left>
+      <right style="thin">
+        <color indexed="64"/>
+      </right>
+      <top style="thin">
+        <color indexed="64"/>
+      </top>
+      <bottom/>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="medium">
+        <color rgb="FF000000"/>
+      </left>
+      <right style="thin">
+        <color rgb="FF000000"/>
+      </right>
+      <top style="thin">
+        <color rgb="FF000000"/>
+      </top>
+      <bottom style="thin">
+        <color rgb="FF000000"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
       <left style="thin">
         <color rgb="FF000000"/>
       </left>
+      <right style="medium">
+        <color rgb="FF000000"/>
+      </right>
+      <top style="thin">
+        <color rgb="FF000000"/>
+      </top>
+      <bottom style="thin">
+        <color rgb="FF000000"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="medium">
+        <color rgb="FF000000"/>
+      </left>
       <right style="thin">
         <color rgb="FF000000"/>
       </right>
       <top style="thin">
         <color rgb="FF000000"/>
       </top>
-      <bottom/>
-      <diagonal/>
-    </border>
-    <border>
-      <left style="medium">
+      <bottom style="medium">
+        <color rgb="FF000000"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="thin">
         <color rgb="FF000000"/>
       </left>
       <right style="thin">
-        <color indexed="64"/>
+        <color rgb="FF000000"/>
       </right>
       <top style="thin">
-        <color indexed="64"/>
-      </top>
-      <bottom style="thin">
-        <color indexed="64"/>
+        <color rgb="FF000000"/>
+      </top>
+      <bottom style="medium">
+        <color rgb="FF000000"/>
       </bottom>
       <diagonal/>
     </border>
     <border>
       <left style="thin">
-        <color indexed="64"/>
+        <color rgb="FF000000"/>
       </left>
       <right style="medium">
         <color rgb="FF000000"/>
       </right>
-      <top/>
-      <bottom/>
-      <diagonal/>
-    </border>
-    <border>
-      <left style="medium">
-        <color indexed="64"/>
-      </left>
-      <right style="thin">
-        <color indexed="64"/>
-      </right>
       <top style="thin">
-        <color indexed="64"/>
-      </top>
-      <bottom/>
-      <diagonal/>
-    </border>
-    <border>
-      <left style="thin">
-        <color indexed="64"/>
-      </left>
-      <right style="medium">
-        <color indexed="64"/>
-      </right>
-      <top style="thin">
-        <color indexed="64"/>
-      </top>
-      <bottom/>
-      <diagonal/>
-    </border>
-    <border>
-      <left style="medium">
-        <color rgb="FF000000"/>
-      </left>
-      <right style="thin">
-        <color indexed="64"/>
-      </right>
-      <top style="thin">
-        <color indexed="64"/>
-      </top>
-      <bottom/>
-      <diagonal/>
-    </border>
-    <border>
-      <left style="medium">
-        <color rgb="FF000000"/>
-      </left>
-      <right style="thin">
-        <color rgb="FF000000"/>
-      </right>
-      <top style="medium">
-        <color rgb="FF000000"/>
-      </top>
-      <bottom style="thin">
-        <color rgb="FF000000"/>
-      </bottom>
-      <diagonal/>
-    </border>
-    <border>
-      <left style="thin">
-        <color rgb="FF000000"/>
-      </left>
-      <right style="thin">
-        <color rgb="FF000000"/>
-      </right>
-      <top style="medium">
-        <color rgb="FF000000"/>
-      </top>
-      <bottom style="thin">
-        <color rgb="FF000000"/>
-      </bottom>
-      <diagonal/>
-    </border>
-    <border>
-      <left style="thin">
-        <color rgb="FF000000"/>
-      </left>
-      <right style="medium">
-        <color rgb="FF000000"/>
-      </right>
-      <top style="medium">
-        <color rgb="FF000000"/>
-      </top>
-      <bottom style="thin">
-        <color rgb="FF000000"/>
-      </bottom>
-      <diagonal/>
-    </border>
-    <border>
-      <left style="medium">
-        <color rgb="FF000000"/>
-      </left>
-      <right style="thin">
-        <color rgb="FF000000"/>
-      </right>
-      <top style="thin">
-        <color rgb="FF000000"/>
-      </top>
-      <bottom style="thin">
-        <color rgb="FF000000"/>
-      </bottom>
-      <diagonal/>
-    </border>
-    <border>
-      <left style="thin">
-        <color rgb="FF000000"/>
-      </left>
-      <right style="medium">
-        <color rgb="FF000000"/>
-      </right>
-      <top style="thin">
-        <color rgb="FF000000"/>
-      </top>
-      <bottom style="thin">
-        <color rgb="FF000000"/>
-      </bottom>
-      <diagonal/>
-    </border>
-    <border>
-      <left style="medium">
-        <color rgb="FF000000"/>
-      </left>
-      <right style="thin">
-        <color rgb="FF000000"/>
-      </right>
-      <top style="thin">
         <color rgb="FF000000"/>
       </top>
       <bottom style="medium">
         <color rgb="FF000000"/>
-      </bottom>
-      <diagonal/>
-    </border>
-    <border>
-      <left style="thin">
-        <color rgb="FF000000"/>
-      </left>
-      <right style="thin">
-        <color rgb="FF000000"/>
-      </right>
-      <top style="thin">
-        <color rgb="FF000000"/>
-      </top>
-      <bottom style="medium">
-        <color rgb="FF000000"/>
-      </bottom>
-      <diagonal/>
-    </border>
-    <border>
-      <left style="thin">
-        <color rgb="FF000000"/>
-      </left>
-      <right style="medium">
-        <color rgb="FF000000"/>
-      </right>
-      <top style="thin">
-        <color rgb="FF000000"/>
-      </top>
-      <bottom style="medium">
-        <color rgb="FF000000"/>
-      </bottom>
-      <diagonal/>
-    </border>
-    <border>
-      <left style="medium">
-        <color rgb="FF000000"/>
-      </left>
-      <right style="thin">
-        <color rgb="FF000000"/>
-      </right>
-      <top style="thin">
-        <color rgb="FF000000"/>
-      </top>
-      <bottom/>
-      <diagonal/>
-    </border>
-    <border>
-      <left style="thin">
-        <color rgb="FF000000"/>
-      </left>
-      <right style="medium">
-        <color rgb="FF000000"/>
-      </right>
-      <top style="thin">
-        <color rgb="FF000000"/>
-      </top>
-      <bottom/>
-      <diagonal/>
-    </border>
-    <border>
-      <left style="medium">
-        <color rgb="FF000000"/>
-      </left>
-      <right style="thin">
-        <color indexed="64"/>
-      </right>
-      <top/>
-      <bottom style="thin">
-        <color indexed="64"/>
-      </bottom>
-      <diagonal/>
-    </border>
-    <border>
-      <left style="thin">
-        <color indexed="64"/>
-      </left>
-      <right style="thin">
-        <color indexed="64"/>
-      </right>
-      <top/>
-      <bottom style="thin">
-        <color indexed="64"/>
       </bottom>
       <diagonal/>
     </border>
@@ -868,153 +718,408 @@
       </bottom>
       <diagonal/>
     </border>
+    <border>
+      <left style="thin">
+        <color indexed="64"/>
+      </left>
+      <right style="medium">
+        <color indexed="64"/>
+      </right>
+      <top style="thin">
+        <color indexed="64"/>
+      </top>
+      <bottom style="medium">
+        <color indexed="64"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="medium">
+        <color rgb="FF000000"/>
+      </left>
+      <right style="thin">
+        <color rgb="FF000000"/>
+      </right>
+      <top/>
+      <bottom style="thin">
+        <color rgb="FF000000"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="thin">
+        <color rgb="FF000000"/>
+      </left>
+      <right style="thin">
+        <color rgb="FF000000"/>
+      </right>
+      <top/>
+      <bottom style="thin">
+        <color rgb="FF000000"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="thin">
+        <color rgb="FF000000"/>
+      </left>
+      <right style="medium">
+        <color rgb="FF000000"/>
+      </right>
+      <top/>
+      <bottom style="thin">
+        <color rgb="FF000000"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="medium">
+        <color indexed="64"/>
+      </left>
+      <right style="thin">
+        <color rgb="FF000000"/>
+      </right>
+      <top style="medium">
+        <color indexed="64"/>
+      </top>
+      <bottom style="thin">
+        <color rgb="FF000000"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="thin">
+        <color rgb="FF000000"/>
+      </left>
+      <right style="thin">
+        <color rgb="FF000000"/>
+      </right>
+      <top style="medium">
+        <color indexed="64"/>
+      </top>
+      <bottom style="thin">
+        <color rgb="FF000000"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="thin">
+        <color rgb="FF000000"/>
+      </left>
+      <right style="medium">
+        <color indexed="64"/>
+      </right>
+      <top style="medium">
+        <color indexed="64"/>
+      </top>
+      <bottom style="thin">
+        <color rgb="FF000000"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="medium">
+        <color indexed="64"/>
+      </left>
+      <right style="thin">
+        <color rgb="FF000000"/>
+      </right>
+      <top style="thin">
+        <color rgb="FF000000"/>
+      </top>
+      <bottom style="thin">
+        <color rgb="FF000000"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="thin">
+        <color rgb="FF000000"/>
+      </left>
+      <right style="medium">
+        <color indexed="64"/>
+      </right>
+      <top style="thin">
+        <color rgb="FF000000"/>
+      </top>
+      <bottom style="thin">
+        <color rgb="FF000000"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="medium">
+        <color indexed="64"/>
+      </left>
+      <right style="thin">
+        <color rgb="FF000000"/>
+      </right>
+      <top style="thin">
+        <color rgb="FF000000"/>
+      </top>
+      <bottom style="medium">
+        <color indexed="64"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="thin">
+        <color rgb="FF000000"/>
+      </left>
+      <right style="thin">
+        <color rgb="FF000000"/>
+      </right>
+      <top style="thin">
+        <color rgb="FF000000"/>
+      </top>
+      <bottom style="medium">
+        <color indexed="64"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="thin">
+        <color rgb="FF000000"/>
+      </left>
+      <right style="medium">
+        <color indexed="64"/>
+      </right>
+      <top style="thin">
+        <color rgb="FF000000"/>
+      </top>
+      <bottom style="medium">
+        <color indexed="64"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="medium">
+        <color indexed="64"/>
+      </left>
+      <right/>
+      <top style="medium">
+        <color indexed="64"/>
+      </top>
+      <bottom/>
+      <diagonal/>
+    </border>
+    <border>
+      <left/>
+      <right/>
+      <top style="medium">
+        <color indexed="64"/>
+      </top>
+      <bottom/>
+      <diagonal/>
+    </border>
+    <border>
+      <left/>
+      <right style="medium">
+        <color indexed="64"/>
+      </right>
+      <top style="medium">
+        <color indexed="64"/>
+      </top>
+      <bottom/>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="medium">
+        <color indexed="64"/>
+      </left>
+      <right/>
+      <top/>
+      <bottom style="medium">
+        <color indexed="64"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left/>
+      <right style="medium">
+        <color indexed="64"/>
+      </right>
+      <top/>
+      <bottom style="medium">
+        <color indexed="64"/>
+      </bottom>
+      <diagonal/>
+    </border>
   </borders>
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="49">
+  <cellXfs count="59">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="2" borderId="36" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="2" borderId="18" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="2" borderId="37" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="7" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="5" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="17" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="20" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="21" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="8" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="8" fillId="0" borderId="7" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="15" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="8" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="16" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="0" borderId="9" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="8" fillId="0" borderId="6" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="0" borderId="17" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="15" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="8" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="16" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="8" fillId="0" borderId="20" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="19" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="8" fillId="0" borderId="7" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="0" borderId="25" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="8" fillId="0" borderId="26" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="27" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="0" borderId="28" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="8" fillId="0" borderId="8" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="29" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="top"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
+    <xf numFmtId="0" fontId="7" fillId="0" borderId="30" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="8" fillId="0" borderId="31" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="32" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="top"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="0" borderId="22" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="8" fillId="0" borderId="23" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="24" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="0" borderId="10" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="11" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="0" borderId="12" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="8" fillId="0" borderId="13" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="14" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="0" borderId="0" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="8" fillId="0" borderId="0" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="16" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="19" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="9" fillId="3" borderId="33" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="9" fillId="3" borderId="34" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="10" fillId="0" borderId="35" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1"/>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="4" borderId="0" xfId="0" applyFill="1" applyAlignment="1">
-      <alignment wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="7" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="8" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="6" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="9" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="6" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="16" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="21" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="17" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="19" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="22" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="10" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="14" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="12" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="15" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="18" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="23" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="20" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="17" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="19" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="top"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="24" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="top"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="5" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="13" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="top"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="3" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="6" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="11" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="25" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="7" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="29" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="30" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="26" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="27" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="28" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="32" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="31" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="11" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="27" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="28" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="31" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
@@ -1031,10 +1136,6 @@
     </ext>
   </extLst>
 </styleSheet>
-</file>
-
-<file path=xl/persons/person.xml><?xml version="1.0" encoding="utf-8"?>
-<personList xmlns="http://schemas.microsoft.com/office/spreadsheetml/2018/threadedcomments" xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main"/>
 </file>
 
 <file path=xl/theme/theme1.xml><?xml version="1.0" encoding="utf-8"?>
@@ -1354,488 +1455,492 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{1C09FB89-CCEB-45F1-BEB7-CE1C325C9FC2}">
-  <dimension ref="B1:D65"/>
-  <sheetFormatPr baseColWidth="10" defaultColWidth="11.5546875" defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
+  <dimension ref="B2:D64"/>
+  <sheetFormatPr defaultColWidth="11.5546875" defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
-    <col min="1" max="1" width="0.88671875" customWidth="1"/>
-    <col min="2" max="2" width="27.44140625" customWidth="1"/>
-    <col min="3" max="3" width="48.21875" style="2" customWidth="1"/>
-    <col min="4" max="4" width="54" customWidth="1"/>
+    <col min="1" max="1" width="0.88671875" style="1" customWidth="1"/>
+    <col min="2" max="2" width="23.5546875" style="1" customWidth="1"/>
+    <col min="3" max="3" width="55.88671875" style="2" customWidth="1"/>
+    <col min="4" max="4" width="50.6640625" style="1" customWidth="1"/>
+    <col min="5" max="16384" width="11.5546875" style="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="2:4" ht="3" customHeight="1" x14ac:dyDescent="0.3"/>
-    <row r="2" spans="2:4" ht="48.6" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="B2" s="33" t="s">
+    <row r="2" spans="2:4" ht="3" customHeight="1" thickBot="1" x14ac:dyDescent="0.35"/>
+    <row r="3" spans="2:4" ht="71.400000000000006" customHeight="1" x14ac:dyDescent="0.4">
+      <c r="B3" s="56" t="s">
         <v>0</v>
       </c>
-      <c r="C2" s="33"/>
-      <c r="D2" s="34"/>
-    </row>
-    <row r="3" spans="2:4" s="3" customFormat="1" ht="18" customHeight="1" thickBot="1" x14ac:dyDescent="0.35">
-      <c r="B3" s="32" t="s">
+      <c r="C3" s="57"/>
+      <c r="D3" s="58"/>
+    </row>
+    <row r="4" spans="2:4" s="6" customFormat="1" ht="21.6" customHeight="1" thickBot="1" x14ac:dyDescent="0.35">
+      <c r="B4" s="3" t="s">
         <v>1</v>
       </c>
-      <c r="C3" s="32" t="s">
+      <c r="C4" s="4" t="s">
         <v>2</v>
       </c>
-      <c r="D3" s="32" t="s">
+      <c r="D4" s="5" t="s">
         <v>3</v>
       </c>
     </row>
-    <row r="4" spans="2:4" ht="28.8" x14ac:dyDescent="0.3">
-      <c r="B4" s="19" t="s">
+    <row r="5" spans="2:4" ht="31.2" x14ac:dyDescent="0.3">
+      <c r="B5" s="7" t="s">
         <v>4</v>
       </c>
-      <c r="C4" s="6" t="s">
+      <c r="C5" s="8" t="s">
         <v>5</v>
       </c>
-      <c r="D4" s="29" t="s">
+      <c r="D5" s="9" t="s">
         <v>71</v>
       </c>
     </row>
-    <row r="5" spans="2:4" ht="28.8" x14ac:dyDescent="0.3">
-      <c r="B5" s="20"/>
-      <c r="C5" s="4" t="s">
+    <row r="6" spans="2:4" ht="46.8" x14ac:dyDescent="0.3">
+      <c r="B6" s="10"/>
+      <c r="C6" s="11" t="s">
         <v>6</v>
       </c>
-      <c r="D5" s="30"/>
-    </row>
-    <row r="6" spans="2:4" ht="28.8" x14ac:dyDescent="0.3">
-      <c r="B6" s="20"/>
-      <c r="C6" s="4" t="s">
+      <c r="D6" s="12"/>
+    </row>
+    <row r="7" spans="2:4" ht="46.8" x14ac:dyDescent="0.3">
+      <c r="B7" s="10"/>
+      <c r="C7" s="11" t="s">
         <v>7</v>
       </c>
-      <c r="D6" s="30"/>
-    </row>
-    <row r="7" spans="2:4" ht="43.2" x14ac:dyDescent="0.3">
-      <c r="B7" s="20"/>
-      <c r="C7" s="4" t="s">
+      <c r="D7" s="12"/>
+    </row>
+    <row r="8" spans="2:4" ht="46.8" x14ac:dyDescent="0.3">
+      <c r="B8" s="10"/>
+      <c r="C8" s="11" t="s">
         <v>73</v>
       </c>
-      <c r="D7" s="30"/>
-    </row>
-    <row r="8" spans="2:4" ht="43.2" x14ac:dyDescent="0.3">
-      <c r="B8" s="20"/>
-      <c r="C8" s="4" t="s">
+      <c r="D8" s="12"/>
+    </row>
+    <row r="9" spans="2:4" ht="46.8" x14ac:dyDescent="0.3">
+      <c r="B9" s="10"/>
+      <c r="C9" s="11" t="s">
         <v>8</v>
       </c>
-      <c r="D8" s="30"/>
-    </row>
-    <row r="9" spans="2:4" ht="30" customHeight="1" thickBot="1" x14ac:dyDescent="0.35">
-      <c r="B9" s="21"/>
-      <c r="C9" s="9" t="s">
+      <c r="D9" s="12"/>
+    </row>
+    <row r="10" spans="2:4" ht="30" customHeight="1" thickBot="1" x14ac:dyDescent="0.35">
+      <c r="B10" s="13"/>
+      <c r="C10" s="14" t="s">
         <v>9</v>
       </c>
-      <c r="D9" s="31"/>
-    </row>
-    <row r="10" spans="2:4" ht="28.8" x14ac:dyDescent="0.3">
-      <c r="B10" s="19" t="s">
+      <c r="D10" s="15"/>
+    </row>
+    <row r="11" spans="2:4" ht="30" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="B11" s="16"/>
+      <c r="C11" s="17"/>
+      <c r="D11" s="18"/>
+    </row>
+    <row r="12" spans="2:4" ht="30" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="B12" s="16"/>
+      <c r="C12" s="17"/>
+      <c r="D12" s="18"/>
+    </row>
+    <row r="13" spans="2:4" ht="30" customHeight="1" thickBot="1" x14ac:dyDescent="0.35">
+      <c r="B13" s="16"/>
+      <c r="C13" s="17"/>
+      <c r="D13" s="18"/>
+    </row>
+    <row r="14" spans="2:4" ht="28.8" x14ac:dyDescent="0.3">
+      <c r="B14" s="19" t="s">
         <v>10</v>
       </c>
-      <c r="C10" s="37" t="s">
+      <c r="C14" s="20" t="s">
         <v>11</v>
       </c>
-      <c r="D10" s="46" t="s">
+      <c r="D14" s="21" t="s">
         <v>72</v>
       </c>
     </row>
-    <row r="11" spans="2:4" ht="28.8" x14ac:dyDescent="0.3">
-      <c r="B11" s="20"/>
-      <c r="C11" s="7" t="s">
+    <row r="15" spans="2:4" ht="28.8" x14ac:dyDescent="0.3">
+      <c r="B15" s="22"/>
+      <c r="C15" s="23" t="s">
         <v>12</v>
       </c>
-      <c r="D11" s="47"/>
-    </row>
-    <row r="12" spans="2:4" x14ac:dyDescent="0.3">
-      <c r="B12" s="20"/>
-      <c r="C12" s="7" t="s">
+      <c r="D15" s="24"/>
+    </row>
+    <row r="16" spans="2:4" ht="28.8" x14ac:dyDescent="0.3">
+      <c r="B16" s="22"/>
+      <c r="C16" s="23" t="s">
         <v>13</v>
       </c>
-      <c r="D12" s="47"/>
-    </row>
-    <row r="13" spans="2:4" ht="43.2" x14ac:dyDescent="0.3">
-      <c r="B13" s="20"/>
-      <c r="C13" s="7" t="s">
+      <c r="D16" s="24"/>
+    </row>
+    <row r="17" spans="2:4" ht="43.2" x14ac:dyDescent="0.3">
+      <c r="B17" s="22"/>
+      <c r="C17" s="23" t="s">
         <v>14</v>
       </c>
-      <c r="D13" s="47"/>
-    </row>
-    <row r="14" spans="2:4" ht="28.8" x14ac:dyDescent="0.3">
-      <c r="B14" s="20"/>
-      <c r="C14" s="7" t="s">
+      <c r="D17" s="24"/>
+    </row>
+    <row r="18" spans="2:4" ht="28.8" x14ac:dyDescent="0.3">
+      <c r="B18" s="22"/>
+      <c r="C18" s="23" t="s">
         <v>15</v>
       </c>
-      <c r="D14" s="47"/>
-    </row>
-    <row r="15" spans="2:4" x14ac:dyDescent="0.3">
-      <c r="B15" s="20"/>
-      <c r="C15" s="7" t="s">
+      <c r="D18" s="24"/>
+    </row>
+    <row r="19" spans="2:4" ht="28.8" x14ac:dyDescent="0.3">
+      <c r="B19" s="22"/>
+      <c r="C19" s="23" t="s">
         <v>16</v>
       </c>
-      <c r="D15" s="47"/>
-    </row>
-    <row r="16" spans="2:4" x14ac:dyDescent="0.3">
-      <c r="B16" s="20"/>
-      <c r="C16" s="7" t="s">
+      <c r="D19" s="24"/>
+    </row>
+    <row r="20" spans="2:4" x14ac:dyDescent="0.3">
+      <c r="B20" s="22"/>
+      <c r="C20" s="23" t="s">
         <v>17</v>
       </c>
-      <c r="D16" s="47"/>
-    </row>
-    <row r="17" spans="2:4" ht="28.8" x14ac:dyDescent="0.3">
-      <c r="B17" s="21"/>
-      <c r="C17" s="11" t="s">
+      <c r="D20" s="24"/>
+    </row>
+    <row r="21" spans="2:4" ht="29.4" thickBot="1" x14ac:dyDescent="0.35">
+      <c r="B21" s="25"/>
+      <c r="C21" s="26" t="s">
         <v>18</v>
       </c>
-      <c r="D17" s="47"/>
-    </row>
-    <row r="18" spans="2:4" ht="13.8" customHeight="1" thickBot="1" x14ac:dyDescent="0.35">
-      <c r="B18" s="38"/>
-      <c r="C18" s="39"/>
-      <c r="D18" s="48"/>
-    </row>
-    <row r="19" spans="2:4" ht="37.200000000000003" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="B19" s="19" t="s">
+      <c r="D21" s="24"/>
+    </row>
+    <row r="22" spans="2:4" ht="17.399999999999999" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="B22" s="19" t="s">
         <v>19</v>
       </c>
-      <c r="C19" s="37" t="s">
+      <c r="C22" s="20" t="s">
         <v>20</v>
       </c>
-      <c r="D19" s="41" t="s">
+      <c r="D22" s="28" t="s">
         <v>21</v>
       </c>
     </row>
-    <row r="20" spans="2:4" ht="28.8" x14ac:dyDescent="0.3">
-      <c r="B20" s="20"/>
-      <c r="C20" s="4" t="s">
+    <row r="23" spans="2:4" ht="28.8" x14ac:dyDescent="0.3">
+      <c r="B23" s="22"/>
+      <c r="C23" s="29" t="s">
         <v>22</v>
       </c>
-      <c r="D20" s="42"/>
-    </row>
-    <row r="21" spans="2:4" ht="43.2" x14ac:dyDescent="0.3">
-      <c r="B21" s="20"/>
-      <c r="C21" s="4" t="s">
+      <c r="D23" s="30"/>
+    </row>
+    <row r="24" spans="2:4" ht="43.2" x14ac:dyDescent="0.3">
+      <c r="B24" s="22"/>
+      <c r="C24" s="29" t="s">
         <v>23</v>
       </c>
-      <c r="D21" s="42"/>
-    </row>
-    <row r="22" spans="2:4" ht="28.8" x14ac:dyDescent="0.3">
-      <c r="B22" s="20"/>
-      <c r="C22" s="4" t="s">
+      <c r="D24" s="30"/>
+    </row>
+    <row r="25" spans="2:4" ht="28.8" x14ac:dyDescent="0.3">
+      <c r="B25" s="22"/>
+      <c r="C25" s="29" t="s">
         <v>24</v>
       </c>
-      <c r="D22" s="42"/>
-    </row>
-    <row r="23" spans="2:4" ht="28.8" x14ac:dyDescent="0.3">
-      <c r="B23" s="20"/>
-      <c r="C23" s="4" t="s">
+      <c r="D25" s="30"/>
+    </row>
+    <row r="26" spans="2:4" ht="28.8" x14ac:dyDescent="0.3">
+      <c r="B26" s="22"/>
+      <c r="C26" s="29" t="s">
         <v>25</v>
       </c>
-      <c r="D23" s="42"/>
-    </row>
-    <row r="24" spans="2:4" ht="28.8" x14ac:dyDescent="0.3">
-      <c r="B24" s="20"/>
-      <c r="C24" s="4" t="s">
+      <c r="D26" s="30"/>
+    </row>
+    <row r="27" spans="2:4" ht="28.8" x14ac:dyDescent="0.3">
+      <c r="B27" s="22"/>
+      <c r="C27" s="29" t="s">
         <v>26</v>
       </c>
-      <c r="D24" s="42"/>
-    </row>
-    <row r="25" spans="2:4" ht="28.8" x14ac:dyDescent="0.3">
-      <c r="B25" s="20"/>
-      <c r="C25" s="4" t="s">
+      <c r="D27" s="30"/>
+    </row>
+    <row r="28" spans="2:4" ht="28.8" x14ac:dyDescent="0.3">
+      <c r="B28" s="22"/>
+      <c r="C28" s="29" t="s">
         <v>27</v>
       </c>
-      <c r="D25" s="42"/>
-    </row>
-    <row r="26" spans="2:4" ht="15" thickBot="1" x14ac:dyDescent="0.35">
-      <c r="B26" s="38"/>
-      <c r="C26" s="43" t="s">
+      <c r="D28" s="30"/>
+    </row>
+    <row r="29" spans="2:4" ht="15" thickBot="1" x14ac:dyDescent="0.35">
+      <c r="B29" s="27"/>
+      <c r="C29" s="31" t="s">
         <v>28</v>
       </c>
-      <c r="D26" s="44"/>
-    </row>
-    <row r="27" spans="2:4" ht="28.8" x14ac:dyDescent="0.3">
-      <c r="B27" s="19" t="s">
+      <c r="D29" s="32"/>
+    </row>
+    <row r="30" spans="2:4" ht="28.8" x14ac:dyDescent="0.3">
+      <c r="B30" s="19" t="s">
         <v>29</v>
       </c>
-      <c r="C27" s="6" t="s">
+      <c r="C30" s="33" t="s">
         <v>30</v>
       </c>
-      <c r="D27" s="41" t="s">
+      <c r="D30" s="28" t="s">
         <v>31</v>
       </c>
     </row>
-    <row r="28" spans="2:4" ht="28.8" x14ac:dyDescent="0.3">
-      <c r="B28" s="20"/>
-      <c r="C28" s="4" t="s">
+    <row r="31" spans="2:4" ht="28.8" x14ac:dyDescent="0.3">
+      <c r="B31" s="22"/>
+      <c r="C31" s="29" t="s">
         <v>32</v>
       </c>
-      <c r="D28" s="42"/>
-    </row>
-    <row r="29" spans="2:4" ht="28.8" x14ac:dyDescent="0.3">
-      <c r="B29" s="20"/>
-      <c r="C29" s="4" t="s">
+      <c r="D31" s="30"/>
+    </row>
+    <row r="32" spans="2:4" ht="28.8" x14ac:dyDescent="0.3">
+      <c r="B32" s="22"/>
+      <c r="C32" s="29" t="s">
         <v>33</v>
       </c>
-      <c r="D29" s="42"/>
-    </row>
-    <row r="30" spans="2:4" x14ac:dyDescent="0.3">
-      <c r="B30" s="20"/>
-      <c r="C30" s="4" t="s">
+      <c r="D32" s="30"/>
+    </row>
+    <row r="33" spans="2:4" x14ac:dyDescent="0.3">
+      <c r="B33" s="22"/>
+      <c r="C33" s="29" t="s">
         <v>34</v>
       </c>
-      <c r="D30" s="42"/>
-    </row>
-    <row r="31" spans="2:4" ht="28.8" x14ac:dyDescent="0.3">
-      <c r="B31" s="20"/>
-      <c r="C31" s="4" t="s">
+      <c r="D33" s="30"/>
+    </row>
+    <row r="34" spans="2:4" ht="28.8" x14ac:dyDescent="0.3">
+      <c r="B34" s="22"/>
+      <c r="C34" s="29" t="s">
         <v>35</v>
       </c>
-      <c r="D31" s="42"/>
-    </row>
-    <row r="32" spans="2:4" x14ac:dyDescent="0.3">
-      <c r="B32" s="20"/>
-      <c r="C32" s="4" t="s">
+      <c r="D34" s="30"/>
+    </row>
+    <row r="35" spans="2:4" x14ac:dyDescent="0.3">
+      <c r="B35" s="22"/>
+      <c r="C35" s="29" t="s">
         <v>36</v>
       </c>
-      <c r="D32" s="42"/>
-    </row>
-    <row r="33" spans="2:4" x14ac:dyDescent="0.3">
-      <c r="B33" s="20"/>
-      <c r="C33" s="4" t="s">
+      <c r="D35" s="30"/>
+    </row>
+    <row r="36" spans="2:4" x14ac:dyDescent="0.3">
+      <c r="B36" s="22"/>
+      <c r="C36" s="29" t="s">
         <v>37</v>
       </c>
-      <c r="D33" s="42"/>
-    </row>
-    <row r="34" spans="2:4" ht="28.8" x14ac:dyDescent="0.3">
-      <c r="B34" s="20"/>
-      <c r="C34" s="4" t="s">
+      <c r="D36" s="30"/>
+    </row>
+    <row r="37" spans="2:4" ht="28.8" x14ac:dyDescent="0.3">
+      <c r="B37" s="22"/>
+      <c r="C37" s="29" t="s">
         <v>38</v>
       </c>
-      <c r="D34" s="42"/>
-    </row>
-    <row r="35" spans="2:4" ht="15" thickBot="1" x14ac:dyDescent="0.35">
-      <c r="B35" s="38"/>
-      <c r="C35" s="43" t="s">
+      <c r="D37" s="30"/>
+    </row>
+    <row r="38" spans="2:4" ht="15" thickBot="1" x14ac:dyDescent="0.35">
+      <c r="B38" s="27"/>
+      <c r="C38" s="31" t="s">
         <v>39</v>
       </c>
-      <c r="D35" s="44"/>
-    </row>
-    <row r="36" spans="2:4" ht="43.2" x14ac:dyDescent="0.3">
-      <c r="B36" s="36" t="s">
+      <c r="D38" s="32"/>
+    </row>
+    <row r="39" spans="2:4" ht="28.8" x14ac:dyDescent="0.3">
+      <c r="B39" s="19" t="s">
         <v>40</v>
       </c>
-      <c r="C36" s="40" t="s">
+      <c r="C39" s="33" t="s">
         <v>41</v>
       </c>
-      <c r="D36" s="45" t="s">
+      <c r="D39" s="21" t="s">
         <v>42</v>
       </c>
     </row>
-    <row r="37" spans="2:4" ht="28.8" x14ac:dyDescent="0.3">
-      <c r="B37" s="17"/>
-      <c r="C37" s="4" t="s">
+    <row r="40" spans="2:4" ht="28.8" x14ac:dyDescent="0.3">
+      <c r="B40" s="22"/>
+      <c r="C40" s="29" t="s">
         <v>43</v>
       </c>
-      <c r="D37" s="35"/>
-    </row>
-    <row r="38" spans="2:4" ht="28.8" x14ac:dyDescent="0.3">
-      <c r="B38" s="17"/>
-      <c r="C38" s="4" t="s">
+      <c r="D40" s="54"/>
+    </row>
+    <row r="41" spans="2:4" ht="28.8" x14ac:dyDescent="0.3">
+      <c r="B41" s="22"/>
+      <c r="C41" s="29" t="s">
         <v>44</v>
       </c>
-      <c r="D38" s="35"/>
-    </row>
-    <row r="39" spans="2:4" x14ac:dyDescent="0.3">
-      <c r="B39" s="17"/>
-      <c r="C39" s="4" t="s">
+      <c r="D41" s="54"/>
+    </row>
+    <row r="42" spans="2:4" x14ac:dyDescent="0.3">
+      <c r="B42" s="22"/>
+      <c r="C42" s="29" t="s">
         <v>45</v>
       </c>
-      <c r="D39" s="35"/>
-    </row>
-    <row r="40" spans="2:4" ht="28.8" x14ac:dyDescent="0.3">
-      <c r="B40" s="17"/>
-      <c r="C40" s="4" t="s">
+      <c r="D42" s="54"/>
+    </row>
+    <row r="43" spans="2:4" ht="28.8" x14ac:dyDescent="0.3">
+      <c r="B43" s="22"/>
+      <c r="C43" s="29" t="s">
         <v>46</v>
       </c>
-      <c r="D40" s="35"/>
-    </row>
-    <row r="41" spans="2:4" x14ac:dyDescent="0.3">
-      <c r="B41" s="17"/>
-      <c r="C41" s="4" t="s">
+      <c r="D43" s="54"/>
+    </row>
+    <row r="44" spans="2:4" x14ac:dyDescent="0.3">
+      <c r="B44" s="22"/>
+      <c r="C44" s="29" t="s">
         <v>47</v>
       </c>
-      <c r="D41" s="35"/>
-    </row>
-    <row r="42" spans="2:4" ht="28.8" x14ac:dyDescent="0.3">
-      <c r="B42" s="17"/>
-      <c r="C42" s="4" t="s">
+      <c r="D44" s="54"/>
+    </row>
+    <row r="45" spans="2:4" ht="28.8" x14ac:dyDescent="0.3">
+      <c r="B45" s="22"/>
+      <c r="C45" s="29" t="s">
         <v>48</v>
       </c>
-      <c r="D42" s="35"/>
-    </row>
-    <row r="43" spans="2:4" ht="68.400000000000006" customHeight="1" thickBot="1" x14ac:dyDescent="0.35">
-      <c r="B43" s="18"/>
-      <c r="C43" s="9" t="s">
+      <c r="D45" s="54"/>
+    </row>
+    <row r="46" spans="2:4" ht="25.2" customHeight="1" thickBot="1" x14ac:dyDescent="0.35">
+      <c r="B46" s="27"/>
+      <c r="C46" s="31" t="s">
         <v>49</v>
       </c>
-      <c r="D43" s="35"/>
-    </row>
-    <row r="44" spans="2:4" ht="15.75" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="B44" s="22" t="s">
+      <c r="D46" s="55"/>
+    </row>
+    <row r="47" spans="2:4" ht="43.8" customHeight="1" thickBot="1" x14ac:dyDescent="0.35">
+      <c r="B47" s="51"/>
+      <c r="C47" s="52"/>
+      <c r="D47" s="53"/>
+    </row>
+    <row r="48" spans="2:4" ht="15.75" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="B48" s="34" t="s">
         <v>50</v>
       </c>
-      <c r="C44" s="12" t="s">
+      <c r="C48" s="35" t="s">
         <v>51</v>
       </c>
-      <c r="D44" s="26" t="s">
+      <c r="D48" s="36" t="s">
         <v>52</v>
       </c>
     </row>
-    <row r="45" spans="2:4" ht="15.75" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="B45" s="23"/>
-      <c r="C45" s="8" t="s">
+    <row r="49" spans="2:4" ht="15.75" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="B49" s="37"/>
+      <c r="C49" s="38" t="s">
         <v>53</v>
       </c>
-      <c r="D45" s="27"/>
-    </row>
-    <row r="46" spans="2:4" ht="15.75" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="B46" s="23"/>
-      <c r="C46" s="8" t="s">
+      <c r="D49" s="39"/>
+    </row>
+    <row r="50" spans="2:4" ht="15.75" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="B50" s="37"/>
+      <c r="C50" s="38" t="s">
         <v>54</v>
       </c>
-      <c r="D46" s="27"/>
-    </row>
-    <row r="47" spans="2:4" ht="15.75" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="B47" s="23"/>
-      <c r="C47" s="8" t="s">
+      <c r="D50" s="39"/>
+    </row>
+    <row r="51" spans="2:4" ht="15.75" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="B51" s="37"/>
+      <c r="C51" s="38" t="s">
         <v>55</v>
       </c>
-      <c r="D47" s="27"/>
-    </row>
-    <row r="48" spans="2:4" ht="15.75" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="B48" s="23"/>
-      <c r="C48" s="8" t="s">
+      <c r="D51" s="39"/>
+    </row>
+    <row r="52" spans="2:4" ht="15.75" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="B52" s="37"/>
+      <c r="C52" s="38" t="s">
         <v>56</v>
       </c>
-      <c r="D48" s="27"/>
-    </row>
-    <row r="49" spans="2:4" ht="15.75" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="B49" s="23"/>
-      <c r="C49" s="8" t="s">
+      <c r="D52" s="39"/>
+    </row>
+    <row r="53" spans="2:4" ht="15.75" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="B53" s="37"/>
+      <c r="C53" s="38" t="s">
         <v>57</v>
       </c>
-      <c r="D49" s="27"/>
-    </row>
-    <row r="50" spans="2:4" ht="15.75" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="B50" s="23"/>
-      <c r="C50" s="8" t="s">
+      <c r="D53" s="39"/>
+    </row>
+    <row r="54" spans="2:4" ht="15.75" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="B54" s="37"/>
+      <c r="C54" s="38" t="s">
         <v>58</v>
       </c>
-      <c r="D50" s="27"/>
-    </row>
-    <row r="51" spans="2:4" ht="53.4" customHeight="1" thickBot="1" x14ac:dyDescent="0.35">
-      <c r="B51" s="24"/>
-      <c r="C51" s="10" t="s">
+      <c r="D54" s="39"/>
+    </row>
+    <row r="55" spans="2:4" ht="53.4" customHeight="1" thickBot="1" x14ac:dyDescent="0.35">
+      <c r="B55" s="40"/>
+      <c r="C55" s="41" t="s">
         <v>59</v>
       </c>
-      <c r="D51" s="28"/>
-    </row>
-    <row r="52" spans="2:4" ht="43.2" x14ac:dyDescent="0.3">
-      <c r="B52" s="22" t="s">
+      <c r="D55" s="42"/>
+    </row>
+    <row r="56" spans="2:4" ht="43.2" x14ac:dyDescent="0.3">
+      <c r="B56" s="43" t="s">
         <v>60</v>
       </c>
-      <c r="C52" s="12" t="s">
+      <c r="C56" s="44" t="s">
         <v>61</v>
       </c>
-      <c r="D52" s="14" t="s">
+      <c r="D56" s="45" t="s">
         <v>62</v>
       </c>
     </row>
-    <row r="53" spans="2:4" ht="28.8" x14ac:dyDescent="0.3">
-      <c r="B53" s="23"/>
-      <c r="C53" s="8" t="s">
+    <row r="57" spans="2:4" ht="28.8" x14ac:dyDescent="0.3">
+      <c r="B57" s="46"/>
+      <c r="C57" s="38" t="s">
         <v>63</v>
       </c>
-      <c r="D53" s="15"/>
-    </row>
-    <row r="54" spans="2:4" ht="14.4" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="B54" s="23"/>
-      <c r="C54" s="8" t="s">
+      <c r="D57" s="47"/>
+    </row>
+    <row r="58" spans="2:4" ht="14.4" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="B58" s="46"/>
+      <c r="C58" s="38" t="s">
         <v>64</v>
       </c>
-      <c r="D54" s="15"/>
-    </row>
-    <row r="55" spans="2:4" ht="14.4" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="B55" s="23"/>
-      <c r="C55" s="8" t="s">
+      <c r="D58" s="47"/>
+    </row>
+    <row r="59" spans="2:4" ht="14.4" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="B59" s="46"/>
+      <c r="C59" s="38" t="s">
         <v>65</v>
       </c>
-      <c r="D55" s="15"/>
-    </row>
-    <row r="56" spans="2:4" ht="28.8" x14ac:dyDescent="0.3">
-      <c r="B56" s="23"/>
-      <c r="C56" s="8" t="s">
+      <c r="D59" s="47"/>
+    </row>
+    <row r="60" spans="2:4" ht="28.8" x14ac:dyDescent="0.3">
+      <c r="B60" s="46"/>
+      <c r="C60" s="38" t="s">
         <v>66</v>
       </c>
-      <c r="D56" s="15"/>
-    </row>
-    <row r="57" spans="2:4" ht="28.8" x14ac:dyDescent="0.3">
-      <c r="B57" s="23"/>
-      <c r="C57" s="8" t="s">
+      <c r="D60" s="47"/>
+    </row>
+    <row r="61" spans="2:4" ht="28.8" x14ac:dyDescent="0.3">
+      <c r="B61" s="46"/>
+      <c r="C61" s="38" t="s">
         <v>67</v>
       </c>
-      <c r="D57" s="15"/>
-    </row>
-    <row r="58" spans="2:4" ht="28.8" x14ac:dyDescent="0.3">
-      <c r="B58" s="23"/>
-      <c r="C58" s="8" t="s">
+      <c r="D61" s="47"/>
+    </row>
+    <row r="62" spans="2:4" ht="28.8" x14ac:dyDescent="0.3">
+      <c r="B62" s="46"/>
+      <c r="C62" s="38" t="s">
         <v>68</v>
       </c>
-      <c r="D58" s="15"/>
-    </row>
-    <row r="59" spans="2:4" ht="46.5" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="B59" s="23"/>
-      <c r="C59" s="8" t="s">
+      <c r="D62" s="47"/>
+    </row>
+    <row r="63" spans="2:4" ht="46.5" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="B63" s="46"/>
+      <c r="C63" s="38" t="s">
         <v>69</v>
       </c>
-      <c r="D59" s="15"/>
-    </row>
-    <row r="60" spans="2:4" ht="14.4" customHeight="1" thickBot="1" x14ac:dyDescent="0.35">
-      <c r="B60" s="25"/>
-      <c r="C60" s="13" t="s">
+      <c r="D63" s="47"/>
+    </row>
+    <row r="64" spans="2:4" ht="14.4" customHeight="1" thickBot="1" x14ac:dyDescent="0.35">
+      <c r="B64" s="48"/>
+      <c r="C64" s="49" t="s">
         <v>70</v>
       </c>
-      <c r="D60" s="16"/>
-    </row>
-    <row r="61" spans="2:4" x14ac:dyDescent="0.3">
-      <c r="B61" s="1"/>
-    </row>
-    <row r="62" spans="2:4" x14ac:dyDescent="0.3">
-      <c r="B62" s="1"/>
-    </row>
-    <row r="63" spans="2:4" x14ac:dyDescent="0.3">
-      <c r="B63" s="1"/>
-    </row>
-    <row r="65" spans="3:3" x14ac:dyDescent="0.3">
-      <c r="C65" s="5"/>
+      <c r="D64" s="50"/>
     </row>
   </sheetData>
   <mergeCells count="15">
-    <mergeCell ref="D36:D43"/>
-    <mergeCell ref="D52:D60"/>
-    <mergeCell ref="B10:B18"/>
-    <mergeCell ref="B4:B9"/>
-    <mergeCell ref="B2:D2"/>
-    <mergeCell ref="D4:D9"/>
-    <mergeCell ref="D10:D18"/>
-    <mergeCell ref="D19:D26"/>
-    <mergeCell ref="B19:B26"/>
-    <mergeCell ref="B27:B35"/>
-    <mergeCell ref="B36:B43"/>
-    <mergeCell ref="B44:B51"/>
-    <mergeCell ref="B52:B60"/>
-    <mergeCell ref="D27:D35"/>
-    <mergeCell ref="D44:D51"/>
+    <mergeCell ref="D39:D46"/>
+    <mergeCell ref="D56:D64"/>
+    <mergeCell ref="B14:B21"/>
+    <mergeCell ref="B5:B10"/>
+    <mergeCell ref="B3:D3"/>
+    <mergeCell ref="D5:D10"/>
+    <mergeCell ref="D14:D21"/>
+    <mergeCell ref="D22:D29"/>
+    <mergeCell ref="B22:B29"/>
+    <mergeCell ref="B30:B38"/>
+    <mergeCell ref="B39:B46"/>
+    <mergeCell ref="B48:B55"/>
+    <mergeCell ref="B56:B64"/>
+    <mergeCell ref="D30:D38"/>
+    <mergeCell ref="D48:D55"/>
   </mergeCells>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup paperSize="9" orientation="landscape" r:id="rId1"/>
@@ -1843,15 +1948,6 @@
 </file>
 
 <file path=customXml/item1.xml><?xml version="1.0" encoding="utf-8"?>
-<?mso-contentType ?>
-<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
-  <Display>DocumentLibraryForm</Display>
-  <Edit>DocumentLibraryForm</Edit>
-  <New>DocumentLibraryForm</New>
-</FormTemplates>
-</file>
-
-<file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
 <ct:contentTypeSchema xmlns:ct="http://schemas.microsoft.com/office/2006/metadata/contentType" xmlns:ma="http://schemas.microsoft.com/office/2006/metadata/properties/metaAttributes" ct:_="" ma:_="" ma:contentTypeName="Documento" ma:contentTypeID="0x010100E784CF8FC968FA419D7090138A1C5306" ma:contentTypeVersion="11" ma:contentTypeDescription="Crear nuevo documento." ma:contentTypeScope="" ma:versionID="39eb63ef951cee5fc2d9dfe9464e3a65">
   <xsd:schema xmlns:xsd="http://www.w3.org/2001/XMLSchema" xmlns:xs="http://www.w3.org/2001/XMLSchema" xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:ns2="ed9a2fb8-b6b8-49e0-9782-a1be223650a2" xmlns:ns3="bcf2c21e-7c8c-4aa1-a238-b3a814444400" targetNamespace="http://schemas.microsoft.com/office/2006/metadata/properties" ma:root="true" ma:fieldsID="0c68340d71e68bd9d23afd1fda0793da" ns2:_="" ns3:_="">
     <xsd:import namespace="ed9a2fb8-b6b8-49e0-9782-a1be223650a2"/>
@@ -2046,7 +2142,7 @@
 </ct:contentTypeSchema>
 </file>
 
-<file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
 <p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
   <documentManagement>
     <lcf76f155ced4ddcb4097134ff3c332f xmlns="ed9a2fb8-b6b8-49e0-9782-a1be223650a2">
@@ -2057,15 +2153,16 @@
 </p:properties>
 </file>
 
-<file path=customXml/itemProps1.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{D4363485-739C-4956-9273-4222E47ADF53}">
-  <ds:schemaRefs>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms"/>
-  </ds:schemaRefs>
-</ds:datastoreItem>
+<file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
+<?mso-contentType ?>
+<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
+  <Display>DocumentLibraryForm</Display>
+  <Edit>DocumentLibraryForm</Edit>
+  <New>DocumentLibraryForm</New>
+</FormTemplates>
 </file>
 
-<file path=customXml/itemProps2.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=customXml/itemProps1.xml><?xml version="1.0" encoding="utf-8"?>
 <ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{2DBB4EC0-8E94-420A-AD84-208349C682FF}">
   <ds:schemaRefs>
     <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/contentType"/>
@@ -2084,7 +2181,7 @@
 </ds:datastoreItem>
 </file>
 
-<file path=customXml/itemProps3.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=customXml/itemProps2.xml><?xml version="1.0" encoding="utf-8"?>
 <ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{5D4874EF-51EB-45FD-AD6C-5A85965AAAED}">
   <ds:schemaRefs>
     <ds:schemaRef ds:uri="http://purl.org/dc/terms/"/>
@@ -2099,4 +2196,12 @@
     <ds:schemaRef ds:uri="http://schemas.openxmlformats.org/package/2006/metadata/core-properties"/>
   </ds:schemaRefs>
 </ds:datastoreItem>
+</file>
+
+<file path=customXml/itemProps3.xml><?xml version="1.0" encoding="utf-8"?>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{D4363485-739C-4956-9273-4222E47ADF53}">
+  <ds:schemaRefs>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms"/>
+  </ds:schemaRefs>
+</ds:datastoreItem>
 </file>
</xml_diff>